<commit_message>
feat: Nuevas funcionalidades en base a preguntas sobre horario
</commit_message>
<xml_diff>
--- a/Copia de Creación de Turnos y roles de la semana. CC097.xlsx
+++ b/Copia de Creación de Turnos y roles de la semana. CC097.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Empleados" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Empleados" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="14">
   <si>
     <t>Empleados</t>
   </si>
@@ -37,49 +37,22 @@
     <t>Horas</t>
   </si>
   <si>
-    <t>Adrián Martos</t>
+    <t>Ana Lopez Garcia</t>
   </si>
   <si>
     <t>10:00-14:00 / 16:30-20:30</t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>Jose Peinado</t>
-  </si>
-  <si>
-    <t>Javier Lopez</t>
-  </si>
-  <si>
-    <t>16:30-20:30</t>
+    <t>DESCANSO</t>
   </si>
   <si>
     <t>10:00-14:00</t>
   </si>
   <si>
-    <t>Hilario Pastrana</t>
-  </si>
-  <si>
-    <t>Fran Catena</t>
-  </si>
-  <si>
-    <t>Fran Cervilla</t>
-  </si>
-  <si>
-    <t>Jose Manuel</t>
-  </si>
-  <si>
-    <t>Antonio Ferron</t>
-  </si>
-  <si>
-    <t>Cinthya Suazo</t>
-  </si>
-  <si>
-    <t>María Ruiz</t>
-  </si>
-  <si>
-    <t>Sol Morales</t>
+    <t>10:00-14:00 / 16:30-18:00</t>
+  </si>
+  <si>
+    <t>16:30-18:00</t>
   </si>
 </sst>
 </file>
@@ -173,6 +146,10 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -376,7 +353,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="16.0"/>
+    <col customWidth="1" min="1" max="1" width="17.38"/>
     <col customWidth="1" min="2" max="7" width="25.0"/>
     <col customWidth="1" min="8" max="8" width="6.63"/>
     <col hidden="1" min="9" max="9" width="12.63"/>
@@ -416,97 +393,91 @@
         <v>9</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H2" s="4">
-        <v>40.0</v>
+        <v>32.0</v>
       </c>
       <c r="I2" s="5">
         <v>40.0</v>
       </c>
     </row>
     <row r="3" ht="51.0" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H3" s="4">
-        <v>40.0</v>
+        <v>27.5</v>
       </c>
       <c r="I3" s="5">
         <v>40.0</v>
       </c>
     </row>
     <row r="4" ht="41.25" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="A4" s="2"/>
       <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H4" s="4">
-        <v>32.0</v>
+        <v>18.0</v>
       </c>
       <c r="I4" s="5">
         <v>32.0</v>
       </c>
     </row>
     <row r="5" ht="45.75" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="A5" s="2"/>
       <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>13</v>
@@ -515,181 +486,169 @@
         <v>13</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H5" s="4">
-        <v>32.0</v>
+        <v>17.0</v>
       </c>
       <c r="I5" s="5">
         <v>32.0</v>
       </c>
     </row>
     <row r="6" ht="47.25" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="A6" s="2"/>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H6" s="4">
-        <v>32.0</v>
+        <v>27.0</v>
       </c>
       <c r="I6" s="5">
         <v>32.0</v>
       </c>
     </row>
     <row r="7" ht="43.5" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="A7" s="2"/>
       <c r="B7" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H7" s="4">
-        <v>36.0</v>
+        <v>22.0</v>
       </c>
       <c r="I7" s="5">
         <v>32.0</v>
       </c>
     </row>
     <row r="8" ht="58.5" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A8" s="2"/>
       <c r="B8" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H8" s="4">
-        <v>32.0</v>
+        <v>19.5</v>
       </c>
       <c r="I8" s="5">
         <v>32.0</v>
       </c>
     </row>
     <row r="9" ht="50.25" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="A9" s="2"/>
       <c r="B9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H9" s="4">
-        <v>32.0</v>
+        <v>22.0</v>
       </c>
       <c r="I9" s="5">
         <v>32.0</v>
       </c>
     </row>
     <row r="10" ht="47.25" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="A10" s="2"/>
       <c r="B10" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H10" s="4">
-        <v>28.0</v>
+        <v>25.5</v>
       </c>
       <c r="I10" s="5">
         <v>28.0</v>
       </c>
     </row>
     <row r="11" ht="45.0" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A11" s="2"/>
       <c r="B11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H11" s="6">
         <v>20.0</v>
@@ -699,29 +658,27 @@
       </c>
     </row>
     <row r="12" ht="45.75" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H12" s="7">
-        <v>28.0</v>
+        <v>18.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>